<commit_message>
about to make a destructive edit
attempting to merge the family and misc arrays
</commit_message>
<xml_diff>
--- a/assets/achievements/achievements guide.xlsx
+++ b/assets/achievements/achievements guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsmy\Downloads\bad life simulator\assets\achievements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEDB24E0-D116-4BAE-8077-14F4E2FF2BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4B8440-7C75-44CA-9A9A-7117DF2F4482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="249">
   <si>
     <t>ID</t>
   </si>
@@ -763,6 +763,15 @@
   </si>
   <si>
     <t>Graduate primary school</t>
+  </si>
+  <si>
+    <t>Beyoncé!?</t>
+  </si>
+  <si>
+    <t>Encounter Beyoncé</t>
+  </si>
+  <si>
+    <t>Have a family member that is, at random life generation, named Beyoncé Beyoncé via easter egg</t>
   </si>
 </sst>
 </file>
@@ -1098,7 +1107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.44140625" customWidth="1"/>
@@ -2975,6 +2984,24 @@
       </c>
       <c r="F115" s="2"/>
     </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116" s="2">
+        <v>114</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="F116" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added (i think) ALL prison events
finally. it might not work properly and probably still needs some bugfixing. also, probably fix the random lawyerCostMultipliers generation, as int(round(float(number))) is ugly as hell and terrible programming. thanks.
</commit_message>
<xml_diff>
--- a/assets/achievements/achievements guide.xlsx
+++ b/assets/achievements/achievements guide.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsmy\Downloads\bad life simulator\assets\achievements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4B8440-7C75-44CA-9A9A-7117DF2F4482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0C7B075-6775-48DF-8099-C0495586D364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="251">
   <si>
     <t>ID</t>
   </si>
@@ -291,9 +291,6 @@
     <t>Get a full-time Job</t>
   </si>
   <si>
-    <t>Unemployed</t>
-  </si>
-  <si>
     <t>Quit (or get fired from) a full-time Job</t>
   </si>
   <si>
@@ -772,6 +769,15 @@
   </si>
   <si>
     <t>Have a family member that is, at random life generation, named Beyoncé Beyoncé via easter egg</t>
+  </si>
+  <si>
+    <t>An absolute natural</t>
+  </si>
+  <si>
+    <t>Successfully defend yourself in court without a law degree</t>
+  </si>
+  <si>
+    <t>De-employed</t>
   </si>
 </sst>
 </file>
@@ -1107,7 +1113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.44140625" customWidth="1"/>
@@ -1131,7 +1137,7 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>26</v>
@@ -1275,7 +1281,7 @@
         <v>23</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="3" t="s">
@@ -1304,7 +1310,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>27</v>
@@ -1322,10 +1328,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>217</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>218</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="3" t="s">
@@ -1486,7 +1492,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>50</v>
@@ -1502,7 +1508,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>51</v>
@@ -1521,7 +1527,7 @@
         <v>52</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="3" t="s">
@@ -1600,7 +1606,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>61</v>
@@ -1618,7 +1624,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>62</v>
@@ -1634,14 +1640,14 @@
         <v>30</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>182</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>183</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F32" s="4">
         <v>1000000</v>
@@ -1798,7 +1804,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>81</v>
@@ -1866,10 +1872,10 @@
         <v>44</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>88</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="3" t="s">
@@ -1882,10 +1888,10 @@
         <v>45</v>
       </c>
       <c r="B47" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>91</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="3" t="s">
@@ -1901,7 +1907,7 @@
         <v>41</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="3" t="s">
@@ -1914,13 +1920,13 @@
         <v>47</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="D49" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>95</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>38</v>
@@ -1932,13 +1938,13 @@
         <v>48</v>
       </c>
       <c r="B50" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C50" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="D50" s="3" t="s">
         <v>97</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>98</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>38</v>
@@ -1950,13 +1956,13 @@
         <v>49</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C51" s="3" t="s">
-        <v>100</v>
-      </c>
       <c r="D51" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>49</v>
@@ -1968,10 +1974,10 @@
         <v>50</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="3" t="s">
@@ -1984,10 +1990,10 @@
         <v>51</v>
       </c>
       <c r="B53" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C53" s="3" t="s">
         <v>102</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>103</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="3" t="s">
@@ -2000,10 +2006,10 @@
         <v>52</v>
       </c>
       <c r="B54" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C54" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="3" t="s">
@@ -2016,10 +2022,10 @@
         <v>53</v>
       </c>
       <c r="B55" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C55" s="3" t="s">
         <v>240</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="D55" s="2"/>
       <c r="E55" s="3" t="s">
@@ -2032,10 +2038,10 @@
         <v>54</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="3" t="s">
@@ -2048,10 +2054,10 @@
         <v>55</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="3" t="s">
@@ -2064,10 +2070,10 @@
         <v>56</v>
       </c>
       <c r="B58" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>110</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="3" t="s">
@@ -2080,10 +2086,10 @@
         <v>57</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="3" t="s">
@@ -2096,10 +2102,10 @@
         <v>58</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="3" t="s">
@@ -2111,10 +2117,10 @@
         <v>59</v>
       </c>
       <c r="B61" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C61" s="3" t="s">
         <v>115</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>116</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="3" t="s">
@@ -2127,10 +2133,10 @@
         <v>60</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="3" t="s">
@@ -2142,10 +2148,10 @@
         <v>61</v>
       </c>
       <c r="B63" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C63" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>119</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="3" t="s">
@@ -2158,13 +2164,13 @@
         <v>62</v>
       </c>
       <c r="B64" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="D64" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>122</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>12</v>
@@ -2178,10 +2184,10 @@
         <v>63</v>
       </c>
       <c r="B65" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C65" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>125</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="3" t="s">
@@ -2194,10 +2200,10 @@
         <v>64</v>
       </c>
       <c r="B66" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C66" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="3" t="s">
@@ -2210,10 +2216,10 @@
         <v>65</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C67" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="3" t="s">
@@ -2226,10 +2232,10 @@
         <v>66</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D68" s="2"/>
       <c r="E68" s="3" t="s">
@@ -2242,10 +2248,10 @@
         <v>67</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D69" s="2"/>
       <c r="E69" s="3" t="s">
@@ -2260,10 +2266,10 @@
         <v>68</v>
       </c>
       <c r="B70" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C70" s="3" t="s">
         <v>132</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>133</v>
       </c>
       <c r="D70" s="2"/>
       <c r="E70" s="3" t="s">
@@ -2276,10 +2282,10 @@
         <v>69</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D71" s="2"/>
       <c r="E71" s="3" t="s">
@@ -2292,10 +2298,10 @@
         <v>70</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D72" s="2"/>
       <c r="E72" s="3" t="s">
@@ -2308,10 +2314,10 @@
         <v>71</v>
       </c>
       <c r="B73" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C73" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>140</v>
       </c>
       <c r="D73" s="2"/>
       <c r="E73" s="3" t="s">
@@ -2324,10 +2330,10 @@
         <v>72</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D74" s="2"/>
       <c r="E74" s="3" t="s">
@@ -2340,10 +2346,10 @@
         <v>73</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D75" s="2"/>
       <c r="E75" s="3" t="s">
@@ -2356,10 +2362,10 @@
         <v>74</v>
       </c>
       <c r="B76" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C76" s="3" t="s">
         <v>144</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>145</v>
       </c>
       <c r="D76" s="2"/>
       <c r="E76" s="3" t="s">
@@ -2372,10 +2378,10 @@
         <v>75</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D77" s="2"/>
       <c r="E77" s="3" t="s">
@@ -2388,10 +2394,10 @@
         <v>76</v>
       </c>
       <c r="B78" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C78" s="3" t="s">
         <v>148</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>149</v>
       </c>
       <c r="D78" s="2"/>
       <c r="E78" s="3" t="s">
@@ -2404,13 +2410,13 @@
         <v>77</v>
       </c>
       <c r="B79" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C79" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="D79" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>38</v>
@@ -2422,10 +2428,10 @@
         <v>78</v>
       </c>
       <c r="B80" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C80" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>156</v>
       </c>
       <c r="D80" s="3"/>
       <c r="E80" s="3" t="s">
@@ -2438,10 +2444,10 @@
         <v>79</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D81" s="2"/>
       <c r="E81" s="3" t="s">
@@ -2454,10 +2460,10 @@
         <v>80</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D82" s="2"/>
       <c r="E82" s="3" t="s">
@@ -2470,10 +2476,10 @@
         <v>81</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D83" s="2"/>
       <c r="E83" s="3" t="s">
@@ -2486,10 +2492,10 @@
         <v>82</v>
       </c>
       <c r="B84" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C84" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>164</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>12</v>
@@ -2500,10 +2506,10 @@
         <v>83</v>
       </c>
       <c r="B85" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C85" s="3" t="s">
         <v>165</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>166</v>
       </c>
       <c r="D85" s="2"/>
       <c r="E85" s="3" t="s">
@@ -2516,10 +2522,10 @@
         <v>84</v>
       </c>
       <c r="B86" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C86" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>170</v>
       </c>
       <c r="D86" s="2"/>
       <c r="E86" s="3" t="s">
@@ -2532,10 +2538,10 @@
         <v>85</v>
       </c>
       <c r="B87" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C87" s="3" t="s">
         <v>171</v>
-      </c>
-      <c r="C87" s="3" t="s">
-        <v>172</v>
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="3" t="s">
@@ -2548,10 +2554,10 @@
         <v>86</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D88" s="2"/>
       <c r="E88" s="3" t="s">
@@ -2564,10 +2570,10 @@
         <v>87</v>
       </c>
       <c r="B89" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C89" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="D89" s="2"/>
       <c r="E89" s="3" t="s">
@@ -2580,14 +2586,14 @@
         <v>88</v>
       </c>
       <c r="B90" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C90" s="3" t="s">
         <v>178</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>179</v>
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
@@ -2595,10 +2601,10 @@
         <v>89</v>
       </c>
       <c r="B91" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C91" s="3" t="s">
         <v>184</v>
-      </c>
-      <c r="C91" s="3" t="s">
-        <v>185</v>
       </c>
       <c r="D91" s="2"/>
       <c r="E91" s="3" t="s">
@@ -2611,10 +2617,10 @@
         <v>90</v>
       </c>
       <c r="B92" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C92" s="3" t="s">
         <v>186</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>187</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>12</v>
@@ -2625,10 +2631,10 @@
         <v>91</v>
       </c>
       <c r="B93" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C93" s="3" t="s">
         <v>188</v>
-      </c>
-      <c r="C93" s="3" t="s">
-        <v>189</v>
       </c>
       <c r="D93" s="2"/>
       <c r="E93" s="3" t="s">
@@ -2641,10 +2647,10 @@
         <v>92</v>
       </c>
       <c r="B94" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="C94" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>193</v>
       </c>
       <c r="D94" s="2"/>
       <c r="E94" s="3" t="s">
@@ -2657,10 +2663,10 @@
         <v>93</v>
       </c>
       <c r="B95" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C95" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="C95" s="3" t="s">
-        <v>195</v>
       </c>
       <c r="D95" s="2"/>
       <c r="E95" s="3" t="s">
@@ -2673,10 +2679,10 @@
         <v>94</v>
       </c>
       <c r="B96" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C96" s="3" t="s">
         <v>196</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>197</v>
       </c>
       <c r="D96" s="2"/>
       <c r="E96" s="3" t="s">
@@ -2689,10 +2695,10 @@
         <v>95</v>
       </c>
       <c r="B97" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C97" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>199</v>
       </c>
       <c r="D97" s="2"/>
       <c r="E97" s="3" t="s">
@@ -2705,10 +2711,10 @@
         <v>96</v>
       </c>
       <c r="B98" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C98" s="3" t="s">
         <v>200</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>201</v>
       </c>
       <c r="D98" s="2"/>
       <c r="E98" s="3" t="s">
@@ -2721,10 +2727,10 @@
         <v>97</v>
       </c>
       <c r="B99" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C99" s="3" t="s">
         <v>202</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>203</v>
       </c>
       <c r="D99" s="2"/>
       <c r="E99" s="3" t="s">
@@ -2737,10 +2743,10 @@
         <v>98</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D100" s="2"/>
       <c r="E100" s="3" t="s">
@@ -2753,10 +2759,10 @@
         <v>99</v>
       </c>
       <c r="B101" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C101" s="3" t="s">
         <v>205</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>206</v>
       </c>
       <c r="D101" s="2"/>
       <c r="E101" s="3" t="s">
@@ -2769,10 +2775,10 @@
         <v>100</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D102" s="2"/>
       <c r="E102" s="3" t="s">
@@ -2785,10 +2791,10 @@
         <v>101</v>
       </c>
       <c r="B103" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="C103" s="3" t="s">
         <v>209</v>
-      </c>
-      <c r="C103" s="3" t="s">
-        <v>210</v>
       </c>
       <c r="D103" s="2"/>
       <c r="E103" s="3" t="s">
@@ -2801,10 +2807,10 @@
         <v>102</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D104" s="2"/>
       <c r="E104" s="3" t="s">
@@ -2817,10 +2823,10 @@
         <v>103</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D105" s="2"/>
       <c r="E105" s="3" t="s">
@@ -2833,13 +2839,13 @@
         <v>104</v>
       </c>
       <c r="B106" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C106" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="C106" s="3" t="s">
-        <v>221</v>
-      </c>
       <c r="E106" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
@@ -2847,10 +2853,10 @@
         <v>105</v>
       </c>
       <c r="B107" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C107" s="3" t="s">
         <v>222</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>223</v>
       </c>
       <c r="D107" s="2"/>
       <c r="E107" s="3" t="s">
@@ -2863,10 +2869,10 @@
         <v>106</v>
       </c>
       <c r="B108" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="C108" s="3" t="s">
         <v>225</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>226</v>
       </c>
       <c r="E108" s="3" t="s">
         <v>7</v>
@@ -2877,10 +2883,10 @@
         <v>107</v>
       </c>
       <c r="B109" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C109" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>228</v>
       </c>
       <c r="D109" s="2"/>
       <c r="E109" s="3" t="s">
@@ -2893,10 +2899,10 @@
         <v>108</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D110" s="2"/>
       <c r="E110" s="3" t="s">
@@ -2909,10 +2915,10 @@
         <v>109</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D111" s="2"/>
       <c r="E111" s="3" t="s">
@@ -2925,10 +2931,10 @@
         <v>110</v>
       </c>
       <c r="B112" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C112" s="3" t="s">
         <v>231</v>
-      </c>
-      <c r="C112" s="3" t="s">
-        <v>232</v>
       </c>
       <c r="D112" s="2"/>
       <c r="E112" s="3" t="s">
@@ -2941,10 +2947,10 @@
         <v>111</v>
       </c>
       <c r="B113" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C113" s="3" t="s">
         <v>235</v>
-      </c>
-      <c r="C113" s="3" t="s">
-        <v>236</v>
       </c>
       <c r="D113" s="2"/>
       <c r="E113" s="3" t="s">
@@ -2957,10 +2963,10 @@
         <v>112</v>
       </c>
       <c r="B114" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C114" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="C114" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="D114" s="2"/>
       <c r="E114" s="3" t="s">
@@ -2973,10 +2979,10 @@
         <v>113</v>
       </c>
       <c r="B115" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C115" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="C115" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="D115" s="2"/>
       <c r="E115" s="3" t="s">
@@ -2989,18 +2995,34 @@
         <v>114</v>
       </c>
       <c r="B116" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="C116" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="C116" s="3" t="s">
+      <c r="D116" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D116" s="2" t="s">
+      <c r="E116" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F116" s="2"/>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A117" s="2">
+        <v>115</v>
+      </c>
+      <c r="B117" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="E116" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="F116" s="2"/>
+      <c r="C117" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D117" s="2"/>
+      <c r="E117" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F117" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>